<commit_message>
Parent progress with Focus next; NVR why-wrong notes and text options; updated pages spreadsheet
</commit_message>
<xml_diff>
--- a/docs/SIGQS-pages.xlsx
+++ b/docs/SIGQS-pages.xlsx
@@ -12,8 +12,8 @@
     <sheet name="API Routes" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Pages'!$A$1:$F$32</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'API Routes'!$A$1:$G$28</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Pages'!$A$1:$F$33</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'API Routes'!$A$1:$G$31</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -497,7 +497,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated from src/app on 2026-10-18.</t>
+          <t>Generated from src/app on 2026-10-18; updated 2026-10-18.</t>
         </is>
       </c>
     </row>
@@ -609,7 +609,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F32"/>
+  <dimension ref="A1:F33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -862,7 +862,7 @@
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>Subject chooser: one card per subject (English, Maths, Verbal, Non-Verbal).</t>
+          <t>Subject chooser: one card per subject (English, Maths, Verbal, Non-Verbal), with a 'Your focus this week' card listing topics the parent set.</t>
         </is>
       </c>
       <c r="E8" s="8" t="inlineStr">
@@ -1140,7 +1140,7 @@
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>/dashboard/[yearId]/[subjectId]</t>
+          <t>/dashboard/focus/[focusId]</t>
         </is>
       </c>
       <c r="C17" s="7" t="inlineStr">
@@ -1150,17 +1150,17 @@
       </c>
       <c r="D17" s="7" t="inlineStr">
         <is>
-          <t>Old year/subject listing; now only redirects to the subject page.</t>
-        </is>
-      </c>
-      <c r="E17" s="9" t="inlineStr">
-        <is>
-          <t>Legacy redirect</t>
+          <t>Start button for an English focus topic: picks a comprehension rich in that question type and opens a round of only those questions.</t>
+        </is>
+      </c>
+      <c r="E17" s="8" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
       <c r="F17" s="7" t="inlineStr">
         <is>
-          <t>src/app/dashboard/[yearId]/[subjectId]/page.tsx</t>
+          <t>src/app/dashboard/focus/[focusId]/page.tsx</t>
         </is>
       </c>
     </row>
@@ -1172,7 +1172,7 @@
       </c>
       <c r="B18" s="7" t="inlineStr">
         <is>
-          <t>/quiz/[compId]</t>
+          <t>/dashboard/[yearId]/[subjectId]</t>
         </is>
       </c>
       <c r="C18" s="7" t="inlineStr">
@@ -1182,17 +1182,17 @@
       </c>
       <c r="D18" s="7" t="inlineStr">
         <is>
-          <t>English comprehension quiz: passage and questions side by side.</t>
-        </is>
-      </c>
-      <c r="E18" s="8" t="inlineStr">
-        <is>
-          <t>Active</t>
+          <t>Old year/subject listing; now only redirects to the subject page.</t>
+        </is>
+      </c>
+      <c r="E18" s="9" t="inlineStr">
+        <is>
+          <t>Legacy redirect</t>
         </is>
       </c>
       <c r="F18" s="7" t="inlineStr">
         <is>
-          <t>src/app/quiz/[compId]/page.tsx</t>
+          <t>src/app/dashboard/[yearId]/[subjectId]/page.tsx</t>
         </is>
       </c>
     </row>
@@ -1204,7 +1204,7 @@
       </c>
       <c r="B19" s="7" t="inlineStr">
         <is>
-          <t>/quiz/maths</t>
+          <t>/quiz/[compId]</t>
         </is>
       </c>
       <c r="C19" s="7" t="inlineStr">
@@ -1214,7 +1214,7 @@
       </c>
       <c r="D19" s="7" t="inlineStr">
         <is>
-          <t>Maths quiz round; level and topic line above the question card.</t>
+          <t>English comprehension quiz: passage and questions side by side. With ?type= it asks only one question type (a focus round).</t>
         </is>
       </c>
       <c r="E19" s="8" t="inlineStr">
@@ -1224,7 +1224,7 @@
       </c>
       <c r="F19" s="7" t="inlineStr">
         <is>
-          <t>src/app/quiz/maths/page.tsx</t>
+          <t>src/app/quiz/[compId]/page.tsx</t>
         </is>
       </c>
     </row>
@@ -1236,7 +1236,7 @@
       </c>
       <c r="B20" s="7" t="inlineStr">
         <is>
-          <t>/quiz/vr</t>
+          <t>/quiz/maths</t>
         </is>
       </c>
       <c r="C20" s="7" t="inlineStr">
@@ -1246,7 +1246,7 @@
       </c>
       <c r="D20" s="7" t="inlineStr">
         <is>
-          <t>Verbal Reasoning quiz round; level and topic line above the question card.</t>
+          <t>Maths quiz round; level and topic line above the question card.</t>
         </is>
       </c>
       <c r="E20" s="8" t="inlineStr">
@@ -1256,7 +1256,7 @@
       </c>
       <c r="F20" s="7" t="inlineStr">
         <is>
-          <t>src/app/quiz/vr/page.tsx</t>
+          <t>src/app/quiz/maths/page.tsx</t>
         </is>
       </c>
     </row>
@@ -1268,7 +1268,7 @@
       </c>
       <c r="B21" s="7" t="inlineStr">
         <is>
-          <t>/quiz/nvr</t>
+          <t>/quiz/vr</t>
         </is>
       </c>
       <c r="C21" s="7" t="inlineStr">
@@ -1278,7 +1278,7 @@
       </c>
       <c r="D21" s="7" t="inlineStr">
         <is>
-          <t>Non-Verbal Reasoning quiz round with figure options.</t>
+          <t>Verbal Reasoning quiz round; level and topic line above the question card.</t>
         </is>
       </c>
       <c r="E21" s="8" t="inlineStr">
@@ -1288,29 +1288,29 @@
       </c>
       <c r="F21" s="7" t="inlineStr">
         <is>
-          <t>src/app/quiz/nvr/page.tsx</t>
+          <t>src/app/quiz/vr/page.tsx</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
         <is>
-          <t>Parent</t>
+          <t>Student</t>
         </is>
       </c>
       <c r="B22" s="7" t="inlineStr">
         <is>
-          <t>/parent</t>
+          <t>/quiz/nvr</t>
         </is>
       </c>
       <c r="C22" s="7" t="inlineStr">
         <is>
-          <t>Parent</t>
+          <t>Student</t>
         </is>
       </c>
       <c r="D22" s="7" t="inlineStr">
         <is>
-          <t>Parent home after login: list of children, what is unlocked, subscription status.</t>
+          <t>Non-Verbal Reasoning quiz round with figure options.</t>
         </is>
       </c>
       <c r="E22" s="8" t="inlineStr">
@@ -1320,7 +1320,7 @@
       </c>
       <c r="F22" s="7" t="inlineStr">
         <is>
-          <t>src/app/parent/page.tsx</t>
+          <t>src/app/quiz/nvr/page.tsx</t>
         </is>
       </c>
     </row>
@@ -1332,7 +1332,7 @@
       </c>
       <c r="B23" s="7" t="inlineStr">
         <is>
-          <t>/parent/kids</t>
+          <t>/parent</t>
         </is>
       </c>
       <c r="C23" s="7" t="inlineStr">
@@ -1342,7 +1342,7 @@
       </c>
       <c r="D23" s="7" t="inlineStr">
         <is>
-          <t>Kids Profile: every child on the account and the form to add another.</t>
+          <t>Parent home after login: How SIGQS Works guide, list of children, what is unlocked, subscription status, time spent.</t>
         </is>
       </c>
       <c r="E23" s="8" t="inlineStr">
@@ -1352,7 +1352,7 @@
       </c>
       <c r="F23" s="7" t="inlineStr">
         <is>
-          <t>src/app/parent/kids/page.tsx</t>
+          <t>src/app/parent/page.tsx</t>
         </is>
       </c>
     </row>
@@ -1364,7 +1364,7 @@
       </c>
       <c r="B24" s="7" t="inlineStr">
         <is>
-          <t>/parent/kids/[studentId]</t>
+          <t>/parent/kids</t>
         </is>
       </c>
       <c r="C24" s="7" t="inlineStr">
@@ -1374,7 +1374,7 @@
       </c>
       <c r="D24" s="7" t="inlineStr">
         <is>
-          <t>Edit one child's profile.</t>
+          <t>Kids Profile: every child on the account and the form to add another.</t>
         </is>
       </c>
       <c r="E24" s="8" t="inlineStr">
@@ -1384,7 +1384,7 @@
       </c>
       <c r="F24" s="7" t="inlineStr">
         <is>
-          <t>src/app/parent/kids/[studentId]/page.tsx</t>
+          <t>src/app/parent/kids/page.tsx</t>
         </is>
       </c>
     </row>
@@ -1396,7 +1396,7 @@
       </c>
       <c r="B25" s="7" t="inlineStr">
         <is>
-          <t>/parent/kids/[studentId]/progress/[subject]</t>
+          <t>/parent/kids/[studentId]</t>
         </is>
       </c>
       <c r="C25" s="7" t="inlineStr">
@@ -1406,7 +1406,7 @@
       </c>
       <c r="D25" s="7" t="inlineStr">
         <is>
-          <t>One child's progress in one subject: time spent, every topic score, latest tests.</t>
+          <t>Edit one child's profile.</t>
         </is>
       </c>
       <c r="E25" s="8" t="inlineStr">
@@ -1416,7 +1416,7 @@
       </c>
       <c r="F25" s="7" t="inlineStr">
         <is>
-          <t>src/app/parent/kids/[studentId]/progress/[subject]/page.tsx</t>
+          <t>src/app/parent/kids/[studentId]/page.tsx</t>
         </is>
       </c>
     </row>
@@ -1428,7 +1428,7 @@
       </c>
       <c r="B26" s="7" t="inlineStr">
         <is>
-          <t>/parent/profile</t>
+          <t>/parent/kids/[studentId]/progress/[subject]</t>
         </is>
       </c>
       <c r="C26" s="7" t="inlineStr">
@@ -1438,7 +1438,7 @@
       </c>
       <c r="D26" s="7" t="inlineStr">
         <is>
-          <t>My Profile: the parent's own name, contact and address.</t>
+          <t>One child's progress in one subject: time spent, Focus next (top topics by questions missed, with Practise this), score bars weakest first with 70% target line, trend arrows, English grouped into skill families from src/config/progress.json, latest tests.</t>
         </is>
       </c>
       <c r="E26" s="8" t="inlineStr">
@@ -1448,29 +1448,29 @@
       </c>
       <c r="F26" s="7" t="inlineStr">
         <is>
-          <t>src/app/parent/profile/page.tsx</t>
+          <t>src/app/parent/kids/[studentId]/progress/[subject]/page.tsx</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
         <is>
-          <t>Admin</t>
+          <t>Parent</t>
         </is>
       </c>
       <c r="B27" s="7" t="inlineStr">
         <is>
-          <t>/admin</t>
+          <t>/parent/profile</t>
         </is>
       </c>
       <c r="C27" s="7" t="inlineStr">
         <is>
-          <t>Admin</t>
+          <t>Parent</t>
         </is>
       </c>
       <c r="D27" s="7" t="inlineStr">
         <is>
-          <t>Admin home: links to content and account tools.</t>
+          <t>My Profile: the parent's own name, contact and address.</t>
         </is>
       </c>
       <c r="E27" s="8" t="inlineStr">
@@ -1480,7 +1480,7 @@
       </c>
       <c r="F27" s="7" t="inlineStr">
         <is>
-          <t>src/app/admin/page.tsx</t>
+          <t>src/app/parent/profile/page.tsx</t>
         </is>
       </c>
     </row>
@@ -1492,7 +1492,7 @@
       </c>
       <c r="B28" s="7" t="inlineStr">
         <is>
-          <t>/admin/english</t>
+          <t>/admin</t>
         </is>
       </c>
       <c r="C28" s="7" t="inlineStr">
@@ -1502,7 +1502,7 @@
       </c>
       <c r="D28" s="7" t="inlineStr">
         <is>
-          <t>Manage English comprehensions by level: create, edit, AI-draft, approve.</t>
+          <t>Admin home: links to content and account tools, and Refresh question lists button.</t>
         </is>
       </c>
       <c r="E28" s="8" t="inlineStr">
@@ -1512,7 +1512,7 @@
       </c>
       <c r="F28" s="7" t="inlineStr">
         <is>
-          <t>src/app/admin/english/page.tsx</t>
+          <t>src/app/admin/page.tsx</t>
         </is>
       </c>
     </row>
@@ -1524,7 +1524,7 @@
       </c>
       <c r="B29" s="7" t="inlineStr">
         <is>
-          <t>/admin/nvr</t>
+          <t>/admin/english</t>
         </is>
       </c>
       <c r="C29" s="7" t="inlineStr">
@@ -1534,7 +1534,7 @@
       </c>
       <c r="D29" s="7" t="inlineStr">
         <is>
-          <t>Browse the Non-Verbal question bank by difficulty and topic.</t>
+          <t>Manage English comprehensions by level: create, edit, AI-draft, approve.</t>
         </is>
       </c>
       <c r="E29" s="8" t="inlineStr">
@@ -1544,7 +1544,7 @@
       </c>
       <c r="F29" s="7" t="inlineStr">
         <is>
-          <t>src/app/admin/nvr/page.tsx</t>
+          <t>src/app/admin/english/page.tsx</t>
         </is>
       </c>
     </row>
@@ -1556,7 +1556,7 @@
       </c>
       <c r="B30" s="7" t="inlineStr">
         <is>
-          <t>/admin/nvr/topic</t>
+          <t>/admin/nvr</t>
         </is>
       </c>
       <c r="C30" s="7" t="inlineStr">
@@ -1566,7 +1566,7 @@
       </c>
       <c r="D30" s="7" t="inlineStr">
         <is>
-          <t>Every question in one Non-Verbal topic and level, with the right answer marked and DB ids shown.</t>
+          <t>Browse the Non-Verbal question bank by difficulty and topic.</t>
         </is>
       </c>
       <c r="E30" s="8" t="inlineStr">
@@ -1576,7 +1576,7 @@
       </c>
       <c r="F30" s="7" t="inlineStr">
         <is>
-          <t>src/app/admin/nvr/topic/page.tsx</t>
+          <t>src/app/admin/nvr/page.tsx</t>
         </is>
       </c>
     </row>
@@ -1588,7 +1588,7 @@
       </c>
       <c r="B31" s="7" t="inlineStr">
         <is>
-          <t>/admin/parent-password</t>
+          <t>/admin/nvr/topic</t>
         </is>
       </c>
       <c r="C31" s="7" t="inlineStr">
@@ -1598,7 +1598,7 @@
       </c>
       <c r="D31" s="7" t="inlineStr">
         <is>
-          <t>Reset a parent's password.</t>
+          <t>Every question in one Non-Verbal topic and level, with the right answer marked and DB ids shown.</t>
         </is>
       </c>
       <c r="E31" s="8" t="inlineStr">
@@ -1608,7 +1608,7 @@
       </c>
       <c r="F31" s="7" t="inlineStr">
         <is>
-          <t>src/app/admin/parent-password/page.tsx</t>
+          <t>src/app/admin/nvr/topic/page.tsx</t>
         </is>
       </c>
     </row>
@@ -1620,32 +1620,64 @@
       </c>
       <c r="B32" s="7" t="inlineStr">
         <is>
+          <t>/admin/parent-password</t>
+        </is>
+      </c>
+      <c r="C32" s="7" t="inlineStr">
+        <is>
+          <t>Admin</t>
+        </is>
+      </c>
+      <c r="D32" s="7" t="inlineStr">
+        <is>
+          <t>Reset a parent's password.</t>
+        </is>
+      </c>
+      <c r="E32" s="8" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="F32" s="7" t="inlineStr">
+        <is>
+          <t>src/app/admin/parent-password/page.tsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="7" t="inlineStr">
+        <is>
+          <t>Admin</t>
+        </is>
+      </c>
+      <c r="B33" s="7" t="inlineStr">
+        <is>
           <t>/admin/admin-password</t>
         </is>
       </c>
-      <c r="C32" s="7" t="inlineStr">
+      <c r="C33" s="7" t="inlineStr">
         <is>
           <t>Admin</t>
         </is>
       </c>
-      <c r="D32" s="7" t="inlineStr">
+      <c r="D33" s="7" t="inlineStr">
         <is>
           <t>Reset an admin's password.</t>
         </is>
       </c>
-      <c r="E32" s="8" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-      <c r="F32" s="7" t="inlineStr">
+      <c r="E33" s="8" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="F33" s="7" t="inlineStr">
         <is>
           <t>src/app/admin/admin-password/page.tsx</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F32"/>
+  <autoFilter ref="A1:F33"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1656,7 +1688,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G28"/>
+  <dimension ref="A1:G31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1913,7 +1945,7 @@
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t>One comprehension plus a random round of nine questions.</t>
+          <t>One comprehension plus a random round of nine questions; ?type= limits the round to one question type.</t>
         </is>
       </c>
       <c r="F7" s="8" t="inlineStr">
@@ -2337,12 +2369,12 @@
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
         <is>
-          <t>Billing</t>
+          <t>Parent</t>
         </is>
       </c>
       <c r="B19" s="7" t="inlineStr">
         <is>
-          <t>/api/parent/billing/checkout</t>
+          <t>/api/parent/focus</t>
         </is>
       </c>
       <c r="C19" s="7" t="inlineStr">
@@ -2352,12 +2384,12 @@
       </c>
       <c r="D19" s="7" t="inlineStr">
         <is>
-          <t>Subscribe button</t>
+          <t>Practise this button (progress page)</t>
         </is>
       </c>
       <c r="E19" s="7" t="inlineStr">
         <is>
-          <t>Starts a monthly Stripe subscription for one child.</t>
+          <t>Sets a topic as the child's focus, shown on the child's dashboard.</t>
         </is>
       </c>
       <c r="F19" s="8" t="inlineStr">
@@ -2367,34 +2399,34 @@
       </c>
       <c r="G19" s="7" t="inlineStr">
         <is>
-          <t>src/app/api/parent/billing/checkout/route.ts</t>
+          <t>src/app/api/parent/focus/route.ts</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
         <is>
-          <t>Billing</t>
+          <t>Parent</t>
         </is>
       </c>
       <c r="B20" s="7" t="inlineStr">
         <is>
-          <t>/api/parent/billing/portal</t>
+          <t>/api/parent/focus/[focusId]</t>
         </is>
       </c>
       <c r="C20" s="7" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>PATCH</t>
         </is>
       </c>
       <c r="D20" s="7" t="inlineStr">
         <is>
-          <t>Manage billing button</t>
+          <t>Remove link (progress page)</t>
         </is>
       </c>
       <c r="E20" s="7" t="inlineStr">
         <is>
-          <t>Opens Stripe's billing portal (card, invoices, cancel).</t>
+          <t>Removes a focus from the child's dashboard; the row is kept with clearedAt set.</t>
         </is>
       </c>
       <c r="F20" s="8" t="inlineStr">
@@ -2404,7 +2436,7 @@
       </c>
       <c r="G20" s="7" t="inlineStr">
         <is>
-          <t>src/app/api/parent/billing/portal/route.ts</t>
+          <t>src/app/api/parent/focus/[focusId]/route.ts</t>
         </is>
       </c>
     </row>
@@ -2416,7 +2448,7 @@
       </c>
       <c r="B21" s="7" t="inlineStr">
         <is>
-          <t>/api/stripe/webhook</t>
+          <t>/api/parent/billing/checkout</t>
         </is>
       </c>
       <c r="C21" s="7" t="inlineStr">
@@ -2426,12 +2458,12 @@
       </c>
       <c r="D21" s="7" t="inlineStr">
         <is>
-          <t>Stripe</t>
+          <t>Subscribe button</t>
         </is>
       </c>
       <c r="E21" s="7" t="inlineStr">
         <is>
-          <t>Receives subscription events and updates the child's access.</t>
+          <t>Starts a monthly Stripe subscription for one child.</t>
         </is>
       </c>
       <c r="F21" s="8" t="inlineStr">
@@ -2441,34 +2473,34 @@
       </c>
       <c r="G21" s="7" t="inlineStr">
         <is>
-          <t>src/app/api/stripe/webhook/route.ts</t>
+          <t>src/app/api/parent/billing/checkout/route.ts</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
         <is>
-          <t>Admin</t>
+          <t>Billing</t>
         </is>
       </c>
       <c r="B22" s="7" t="inlineStr">
         <is>
-          <t>/api/admin/english</t>
+          <t>/api/parent/billing/portal</t>
         </is>
       </c>
       <c r="C22" s="7" t="inlineStr">
         <is>
-          <t>GET, POST</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="D22" s="7" t="inlineStr">
         <is>
-          <t>Admin English</t>
+          <t>Manage billing button</t>
         </is>
       </c>
       <c r="E22" s="7" t="inlineStr">
         <is>
-          <t>Lists comprehensions (optionally by year) and creates new ones.</t>
+          <t>Opens Stripe's billing portal (card, invoices, cancel).</t>
         </is>
       </c>
       <c r="F22" s="8" t="inlineStr">
@@ -2478,19 +2510,19 @@
       </c>
       <c r="G22" s="7" t="inlineStr">
         <is>
-          <t>src/app/api/admin/english/route.ts</t>
+          <t>src/app/api/parent/billing/portal/route.ts</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
         <is>
-          <t>Admin</t>
+          <t>Billing</t>
         </is>
       </c>
       <c r="B23" s="7" t="inlineStr">
         <is>
-          <t>/api/admin/english/generate</t>
+          <t>/api/stripe/webhook</t>
         </is>
       </c>
       <c r="C23" s="7" t="inlineStr">
@@ -2500,12 +2532,12 @@
       </c>
       <c r="D23" s="7" t="inlineStr">
         <is>
-          <t>Admin English</t>
+          <t>Stripe</t>
         </is>
       </c>
       <c r="E23" s="7" t="inlineStr">
         <is>
-          <t>Drafts a comprehension with Claude for the admin to review; saves nothing.</t>
+          <t>Receives subscription events and updates the child's access.</t>
         </is>
       </c>
       <c r="F23" s="8" t="inlineStr">
@@ -2515,7 +2547,7 @@
       </c>
       <c r="G23" s="7" t="inlineStr">
         <is>
-          <t>src/app/api/admin/english/generate/route.ts</t>
+          <t>src/app/api/stripe/webhook/route.ts</t>
         </is>
       </c>
     </row>
@@ -2527,12 +2559,12 @@
       </c>
       <c r="B24" s="7" t="inlineStr">
         <is>
-          <t>/api/admin/comps/[compId]</t>
+          <t>/api/admin/english</t>
         </is>
       </c>
       <c r="C24" s="7" t="inlineStr">
         <is>
-          <t>GET, PATCH, DELETE</t>
+          <t>GET, POST</t>
         </is>
       </c>
       <c r="D24" s="7" t="inlineStr">
@@ -2542,7 +2574,7 @@
       </c>
       <c r="E24" s="7" t="inlineStr">
         <is>
-          <t>Reads, edits or removes one comprehension.</t>
+          <t>Lists comprehensions (optionally by year) and creates new ones.</t>
         </is>
       </c>
       <c r="F24" s="8" t="inlineStr">
@@ -2552,7 +2584,7 @@
       </c>
       <c r="G24" s="7" t="inlineStr">
         <is>
-          <t>src/app/api/admin/comps/[compId]/route.ts</t>
+          <t>src/app/api/admin/english/route.ts</t>
         </is>
       </c>
     </row>
@@ -2564,7 +2596,7 @@
       </c>
       <c r="B25" s="7" t="inlineStr">
         <is>
-          <t>/api/admin/comps/[compId]/questions</t>
+          <t>/api/admin/english/generate</t>
         </is>
       </c>
       <c r="C25" s="7" t="inlineStr">
@@ -2579,7 +2611,7 @@
       </c>
       <c r="E25" s="7" t="inlineStr">
         <is>
-          <t>Adds questions to a comprehension.</t>
+          <t>Drafts a comprehension with Claude for the admin to review; saves nothing.</t>
         </is>
       </c>
       <c r="F25" s="8" t="inlineStr">
@@ -2589,7 +2621,7 @@
       </c>
       <c r="G25" s="7" t="inlineStr">
         <is>
-          <t>src/app/api/admin/comps/[compId]/questions/route.ts</t>
+          <t>src/app/api/admin/english/generate/route.ts</t>
         </is>
       </c>
     </row>
@@ -2601,12 +2633,12 @@
       </c>
       <c r="B26" s="7" t="inlineStr">
         <is>
-          <t>/api/admin/comps/[compId]/questions/[questionId]</t>
+          <t>/api/admin/comps/[compId]</t>
         </is>
       </c>
       <c r="C26" s="7" t="inlineStr">
         <is>
-          <t>PATCH, DELETE</t>
+          <t>GET, PATCH, DELETE</t>
         </is>
       </c>
       <c r="D26" s="7" t="inlineStr">
@@ -2616,7 +2648,7 @@
       </c>
       <c r="E26" s="7" t="inlineStr">
         <is>
-          <t>Edits or removes one comprehension question.</t>
+          <t>Reads, edits or removes one comprehension.</t>
         </is>
       </c>
       <c r="F26" s="8" t="inlineStr">
@@ -2626,7 +2658,7 @@
       </c>
       <c r="G26" s="7" t="inlineStr">
         <is>
-          <t>src/app/api/admin/comps/[compId]/questions/[questionId]/route.ts</t>
+          <t>src/app/api/admin/comps/[compId]/route.ts</t>
         </is>
       </c>
     </row>
@@ -2638,22 +2670,22 @@
       </c>
       <c r="B27" s="7" t="inlineStr">
         <is>
-          <t>/api/admin/parent-password</t>
+          <t>/api/admin/comps/[compId]/questions</t>
         </is>
       </c>
       <c r="C27" s="7" t="inlineStr">
         <is>
-          <t>GET, POST</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="D27" s="7" t="inlineStr">
         <is>
-          <t>Admin parent-password page</t>
+          <t>Admin English</t>
         </is>
       </c>
       <c r="E27" s="7" t="inlineStr">
         <is>
-          <t>Lists parents and resets a parent's password.</t>
+          <t>Adds questions to a comprehension.</t>
         </is>
       </c>
       <c r="F27" s="8" t="inlineStr">
@@ -2663,7 +2695,7 @@
       </c>
       <c r="G27" s="7" t="inlineStr">
         <is>
-          <t>src/app/api/admin/parent-password/route.ts</t>
+          <t>src/app/api/admin/comps/[compId]/questions/route.ts</t>
         </is>
       </c>
     </row>
@@ -2675,37 +2707,148 @@
       </c>
       <c r="B28" s="7" t="inlineStr">
         <is>
+          <t>/api/admin/comps/[compId]/questions/[questionId]</t>
+        </is>
+      </c>
+      <c r="C28" s="7" t="inlineStr">
+        <is>
+          <t>PATCH, DELETE</t>
+        </is>
+      </c>
+      <c r="D28" s="7" t="inlineStr">
+        <is>
+          <t>Admin English</t>
+        </is>
+      </c>
+      <c r="E28" s="7" t="inlineStr">
+        <is>
+          <t>Edits or removes one comprehension question.</t>
+        </is>
+      </c>
+      <c r="F28" s="8" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="G28" s="7" t="inlineStr">
+        <is>
+          <t>src/app/api/admin/comps/[compId]/questions/[questionId]/route.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="7" t="inlineStr">
+        <is>
+          <t>Admin</t>
+        </is>
+      </c>
+      <c r="B29" s="7" t="inlineStr">
+        <is>
+          <t>/api/admin/refresh-question-bank</t>
+        </is>
+      </c>
+      <c r="C29" s="7" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="D29" s="7" t="inlineStr">
+        <is>
+          <t>Admin home Refresh now button</t>
+        </is>
+      </c>
+      <c r="E29" s="7" t="inlineStr">
+        <is>
+          <t>Clears the cached Maths, Verbal and Non-Verbal level/topic lists (otherwise flushed daily at 03:00 UK time).</t>
+        </is>
+      </c>
+      <c r="F29" s="8" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="G29" s="7" t="inlineStr">
+        <is>
+          <t>src/app/api/admin/refresh-question-bank/route.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="7" t="inlineStr">
+        <is>
+          <t>Admin</t>
+        </is>
+      </c>
+      <c r="B30" s="7" t="inlineStr">
+        <is>
+          <t>/api/admin/parent-password</t>
+        </is>
+      </c>
+      <c r="C30" s="7" t="inlineStr">
+        <is>
+          <t>GET, POST</t>
+        </is>
+      </c>
+      <c r="D30" s="7" t="inlineStr">
+        <is>
+          <t>Admin parent-password page</t>
+        </is>
+      </c>
+      <c r="E30" s="7" t="inlineStr">
+        <is>
+          <t>Lists parents and resets a parent's password.</t>
+        </is>
+      </c>
+      <c r="F30" s="8" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="G30" s="7" t="inlineStr">
+        <is>
+          <t>src/app/api/admin/parent-password/route.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="7" t="inlineStr">
+        <is>
+          <t>Admin</t>
+        </is>
+      </c>
+      <c r="B31" s="7" t="inlineStr">
+        <is>
           <t>/api/admin/admin-password</t>
         </is>
       </c>
-      <c r="C28" s="7" t="inlineStr">
+      <c r="C31" s="7" t="inlineStr">
         <is>
           <t>GET, POST</t>
         </is>
       </c>
-      <c r="D28" s="7" t="inlineStr">
+      <c r="D31" s="7" t="inlineStr">
         <is>
           <t>Admin admin-password page</t>
         </is>
       </c>
-      <c r="E28" s="7" t="inlineStr">
+      <c r="E31" s="7" t="inlineStr">
         <is>
           <t>Lists admins and resets an admin's password.</t>
         </is>
       </c>
-      <c r="F28" s="8" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-      <c r="G28" s="7" t="inlineStr">
+      <c r="F31" s="8" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="G31" s="7" t="inlineStr">
         <is>
           <t>src/app/api/admin/admin-password/route.ts</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G28"/>
+  <autoFilter ref="A1:G31"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Programmes (Grammar School, GCSE, A-Level) with Preparing for on child forms; updated pages spreadsheet
</commit_message>
<xml_diff>
--- a/docs/SIGQS-pages.xlsx
+++ b/docs/SIGQS-pages.xlsx
@@ -10,10 +10,14 @@
     <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Pages" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="API Routes" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Config Files" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Migrations" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Pages'!$A$1:$F$33</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'API Routes'!$A$1:$G$31</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Pages'!$A$1:$F$34</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'API Routes'!$A$1:$G$33</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Config Files'!$A$1:$D$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Migrations'!$A$1:$C$10</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -490,14 +494,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>SIGQS - pages and API routes</t>
+          <t>SIGQS - pages, API routes, config files and migrations</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated from src/app on 2026-10-18; updated 2026-10-18.</t>
+          <t>Generated from src/app; last updated 2026-10-24.</t>
         </is>
       </c>
     </row>
@@ -609,7 +613,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F33"/>
+  <dimension ref="A1:F34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -702,7 +706,7 @@
       </c>
       <c r="D3" s="7" t="inlineStr">
         <is>
-          <t>Sign-in page with the full SIGQS logo and motto; students, parents and admins all log in here.</t>
+          <t>Sign-in page with the full SIGQS logo and motto; students, parents and admins all log in here. Shows a notice after an inactivity sign-out.</t>
         </is>
       </c>
       <c r="E3" s="8" t="inlineStr">
@@ -734,7 +738,7 @@
       </c>
       <c r="D4" s="7" t="inlineStr">
         <is>
-          <t>Parent sign-up form; parent must accept the Terms &amp; Copyright notice. Children are added later from Kids Profile.</t>
+          <t>Parent sign-up form: name, email, login ID, password and Country (United Kingdom pre-selected). Parent must accept the Terms &amp; Copyright notice. Children are added later from Kids Profile.</t>
         </is>
       </c>
       <c r="E4" s="8" t="inlineStr">
@@ -862,7 +866,7 @@
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>Subject chooser: one card per subject (English, Maths, Verbal, Non-Verbal), with a 'Your focus this week' card listing topics the parent set.</t>
+          <t>Subject chooser: one card per subject (English, Maths, Verbal, Non-Verbal), counting only the child's programme's content, with a 'Your focus this week' card listing topics the parent set.</t>
         </is>
       </c>
       <c r="E8" s="8" t="inlineStr">
@@ -894,7 +898,7 @@
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>English comprehensions banded by difficulty, each with the student's last three scores.</t>
+          <t>English comprehensions in the child's programme, banded by difficulty, each with the student's last three scores.</t>
         </is>
       </c>
       <c r="E9" s="8" t="inlineStr">
@@ -958,7 +962,7 @@
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
-          <t>Maths picker: choose difficulty, then topic and subtopic to start a round.</t>
+          <t>Maths picker for the child's programme: choose difficulty, then topic and subtopic to start a round.</t>
         </is>
       </c>
       <c r="E11" s="8" t="inlineStr">
@@ -1342,7 +1346,7 @@
       </c>
       <c r="D23" s="7" t="inlineStr">
         <is>
-          <t>Parent home after login: How SIGQS Works guide, list of children, what is unlocked, subscription status, time spent.</t>
+          <t>Parent home after login: How SIGQS Works guide, list of children, what is unlocked, time spent. Subscribe button hidden by src/config/billing.json; paid children still show Manage billing.</t>
         </is>
       </c>
       <c r="E23" s="8" t="inlineStr">
@@ -1374,7 +1378,7 @@
       </c>
       <c r="D24" s="7" t="inlineStr">
         <is>
-          <t>Kids Profile: every child on the account and the form to add another.</t>
+          <t>Kids Profile: every child on the account and the form to add another (name, login ID, password, school year, Preparing for, Country).</t>
         </is>
       </c>
       <c r="E24" s="8" t="inlineStr">
@@ -1406,7 +1410,7 @@
       </c>
       <c r="D25" s="7" t="inlineStr">
         <is>
-          <t>Edit one child's profile.</t>
+          <t>Edit one child's profile: name, school year, Preparing for (programme), password, active.</t>
         </is>
       </c>
       <c r="E25" s="8" t="inlineStr">
@@ -1502,7 +1506,7 @@
       </c>
       <c r="D28" s="7" t="inlineStr">
         <is>
-          <t>Admin home: links to content and account tools, and Refresh question lists button.</t>
+          <t>Admin home: links to content and account tools (including Generate English with Claude), and Refresh question lists button.</t>
         </is>
       </c>
       <c r="E28" s="8" t="inlineStr">
@@ -1534,7 +1538,7 @@
       </c>
       <c r="D29" s="7" t="inlineStr">
         <is>
-          <t>Manage English comprehensions by level: create, edit, AI-draft, approve.</t>
+          <t>Manage English comprehensions by level: edit, approve, add questions; link to Generate with Claude.</t>
         </is>
       </c>
       <c r="E29" s="8" t="inlineStr">
@@ -1556,7 +1560,7 @@
       </c>
       <c r="B30" s="7" t="inlineStr">
         <is>
-          <t>/admin/nvr</t>
+          <t>/admin/english/generate</t>
         </is>
       </c>
       <c r="C30" s="7" t="inlineStr">
@@ -1566,7 +1570,7 @@
       </c>
       <c r="D30" s="7" t="inlineStr">
         <is>
-          <t>Browse the Non-Verbal question bank by difficulty and topic.</t>
+          <t>Draft a new English comprehension with Claude: year, level, question count, prompt, up to 3 reference passages and editable copyright guidance. Shows the draft with answers marked; can save it as an unapproved passage.</t>
         </is>
       </c>
       <c r="E30" s="8" t="inlineStr">
@@ -1576,7 +1580,7 @@
       </c>
       <c r="F30" s="7" t="inlineStr">
         <is>
-          <t>src/app/admin/nvr/page.tsx</t>
+          <t>src/app/admin/english/generate/page.tsx</t>
         </is>
       </c>
     </row>
@@ -1588,7 +1592,7 @@
       </c>
       <c r="B31" s="7" t="inlineStr">
         <is>
-          <t>/admin/nvr/topic</t>
+          <t>/admin/nvr</t>
         </is>
       </c>
       <c r="C31" s="7" t="inlineStr">
@@ -1598,7 +1602,7 @@
       </c>
       <c r="D31" s="7" t="inlineStr">
         <is>
-          <t>Every question in one Non-Verbal topic and level, with the right answer marked and DB ids shown.</t>
+          <t>Browse the Non-Verbal question bank by difficulty and topic.</t>
         </is>
       </c>
       <c r="E31" s="8" t="inlineStr">
@@ -1608,7 +1612,7 @@
       </c>
       <c r="F31" s="7" t="inlineStr">
         <is>
-          <t>src/app/admin/nvr/topic/page.tsx</t>
+          <t>src/app/admin/nvr/page.tsx</t>
         </is>
       </c>
     </row>
@@ -1620,7 +1624,7 @@
       </c>
       <c r="B32" s="7" t="inlineStr">
         <is>
-          <t>/admin/parent-password</t>
+          <t>/admin/nvr/topic</t>
         </is>
       </c>
       <c r="C32" s="7" t="inlineStr">
@@ -1630,7 +1634,7 @@
       </c>
       <c r="D32" s="7" t="inlineStr">
         <is>
-          <t>Reset a parent's password.</t>
+          <t>Every question in one Non-Verbal topic and level, with the right answer marked and DB ids shown.</t>
         </is>
       </c>
       <c r="E32" s="8" t="inlineStr">
@@ -1640,7 +1644,7 @@
       </c>
       <c r="F32" s="7" t="inlineStr">
         <is>
-          <t>src/app/admin/parent-password/page.tsx</t>
+          <t>src/app/admin/nvr/topic/page.tsx</t>
         </is>
       </c>
     </row>
@@ -1652,32 +1656,64 @@
       </c>
       <c r="B33" s="7" t="inlineStr">
         <is>
+          <t>/admin/parent-password</t>
+        </is>
+      </c>
+      <c r="C33" s="7" t="inlineStr">
+        <is>
+          <t>Admin</t>
+        </is>
+      </c>
+      <c r="D33" s="7" t="inlineStr">
+        <is>
+          <t>Reset a parent's password.</t>
+        </is>
+      </c>
+      <c r="E33" s="8" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="F33" s="7" t="inlineStr">
+        <is>
+          <t>src/app/admin/parent-password/page.tsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="7" t="inlineStr">
+        <is>
+          <t>Admin</t>
+        </is>
+      </c>
+      <c r="B34" s="7" t="inlineStr">
+        <is>
           <t>/admin/admin-password</t>
         </is>
       </c>
-      <c r="C33" s="7" t="inlineStr">
+      <c r="C34" s="7" t="inlineStr">
         <is>
           <t>Admin</t>
         </is>
       </c>
-      <c r="D33" s="7" t="inlineStr">
+      <c r="D34" s="7" t="inlineStr">
         <is>
           <t>Reset an admin's password.</t>
         </is>
       </c>
-      <c r="E33" s="8" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-      <c r="F33" s="7" t="inlineStr">
+      <c r="E34" s="8" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="F34" s="7" t="inlineStr">
         <is>
           <t>src/app/admin/admin-password/page.tsx</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F33"/>
+  <autoFilter ref="A1:F34"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1688,7 +1724,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G31"/>
+  <dimension ref="A1:G33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1760,7 +1796,7 @@
       </c>
       <c r="E2" s="7" t="inlineStr">
         <is>
-          <t>Checks credentials, starts a session and records the login.</t>
+          <t>Checks credentials, starts a session (token carries the programme) and records the login. Locks a login ID after 8 wrong passwords for 15 min; 30 attempts per network address per 15 min.</t>
         </is>
       </c>
       <c r="F2" s="8" t="inlineStr">
@@ -1834,7 +1870,7 @@
       </c>
       <c r="E4" s="7" t="inlineStr">
         <is>
-          <t>Creates a PARENT account and records terms acceptance.</t>
+          <t>Creates a PARENT account with country and terms acceptance. Limited to 5 sign-ups per network address per hour.</t>
         </is>
       </c>
       <c r="F4" s="8" t="inlineStr">
@@ -1856,7 +1892,7 @@
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>/api/auth/forgot-password</t>
+          <t>/api/auth/keepalive</t>
         </is>
       </c>
       <c r="C5" s="7" t="inlineStr">
@@ -1866,12 +1902,12 @@
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>Forgot-password page</t>
+          <t>Every signed-in page (on activity, at most every 5 min)</t>
         </is>
       </c>
       <c r="E5" s="7" t="inlineStr">
         <is>
-          <t>Emails a reset link; always gives the same answer.</t>
+          <t>Renews the session token while the user is active; re-reads programme and active status. Idle sessions expire after 150 min.</t>
         </is>
       </c>
       <c r="F5" s="8" t="inlineStr">
@@ -1881,7 +1917,7 @@
       </c>
       <c r="G5" s="7" t="inlineStr">
         <is>
-          <t>src/app/api/auth/forgot-password/route.ts</t>
+          <t>src/app/api/auth/keepalive/route.ts</t>
         </is>
       </c>
     </row>
@@ -1893,22 +1929,22 @@
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>/api/auth/reset-password</t>
+          <t>/api/auth/forgot-password</t>
         </is>
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>GET, POST</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>Reset-password page</t>
+          <t>Forgot-password page</t>
         </is>
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
-          <t>GET checks the link is still valid; POST sets the new password.</t>
+          <t>Emails a reset link; always gives the same answer. 5 requests per network address per 15 min.</t>
         </is>
       </c>
       <c r="F6" s="8" t="inlineStr">
@@ -1918,34 +1954,34 @@
       </c>
       <c r="G6" s="7" t="inlineStr">
         <is>
-          <t>src/app/api/auth/reset-password/route.ts</t>
+          <t>src/app/api/auth/forgot-password/route.ts</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>Auth</t>
         </is>
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>/api/comps/[id]</t>
+          <t>/api/auth/reset-password</t>
         </is>
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>GET, POST</t>
         </is>
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>English quiz</t>
+          <t>Reset-password page</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t>One comprehension plus a random round of nine questions; ?type= limits the round to one question type.</t>
+          <t>GET checks the link is still valid; POST sets the new password. 10 per network address per 15 min.</t>
         </is>
       </c>
       <c r="F7" s="8" t="inlineStr">
@@ -1955,34 +1991,34 @@
       </c>
       <c r="G7" s="7" t="inlineStr">
         <is>
-          <t>src/app/api/comps/[id]/route.ts</t>
+          <t>src/app/api/auth/reset-password/route.ts</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>Public</t>
         </is>
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>/api/comps/[id]/submit</t>
+          <t>/api/countries</t>
         </is>
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>English quiz</t>
+          <t>Sign-up page</t>
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
-          <t>Grades and saves an English round.</t>
+          <t>Country list for the drop-downs (code, name, dialling code), United Kingdom first.</t>
         </is>
       </c>
       <c r="F8" s="8" t="inlineStr">
@@ -1992,19 +2028,19 @@
       </c>
       <c r="G8" s="7" t="inlineStr">
         <is>
-          <t>src/app/api/comps/[id]/submit/route.ts</t>
+          <t>src/app/api/countries/route.ts</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t>Maths</t>
+          <t>English</t>
         </is>
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>/api/maths/questions</t>
+          <t>/api/comps/[id]</t>
         </is>
       </c>
       <c r="C9" s="7" t="inlineStr">
@@ -2014,12 +2050,12 @@
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>Maths quiz</t>
+          <t>English quiz</t>
         </is>
       </c>
       <c r="E9" s="7" t="inlineStr">
         <is>
-          <t>Random Maths round for a subtopic/topic and level; answers withheld.</t>
+          <t>One comprehension plus a random round of nine questions; ?type= limits the round to one question type.</t>
         </is>
       </c>
       <c r="F9" s="8" t="inlineStr">
@@ -2029,19 +2065,19 @@
       </c>
       <c r="G9" s="7" t="inlineStr">
         <is>
-          <t>src/app/api/maths/questions/route.ts</t>
+          <t>src/app/api/comps/[id]/route.ts</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t>Maths</t>
+          <t>English</t>
         </is>
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>/api/maths/submit</t>
+          <t>/api/comps/[id]/submit</t>
         </is>
       </c>
       <c r="C10" s="7" t="inlineStr">
@@ -2051,12 +2087,12 @@
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>Maths quiz</t>
+          <t>English quiz</t>
         </is>
       </c>
       <c r="E10" s="7" t="inlineStr">
         <is>
-          <t>Grades and saves a Maths round.</t>
+          <t>Grades and saves an English round; only passages in the student's programme.</t>
         </is>
       </c>
       <c r="F10" s="8" t="inlineStr">
@@ -2066,19 +2102,19 @@
       </c>
       <c r="G10" s="7" t="inlineStr">
         <is>
-          <t>src/app/api/maths/submit/route.ts</t>
+          <t>src/app/api/comps/[id]/submit/route.ts</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t>Verbal</t>
+          <t>Maths</t>
         </is>
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>/api/vr/questions</t>
+          <t>/api/maths/questions</t>
         </is>
       </c>
       <c r="C11" s="7" t="inlineStr">
@@ -2088,12 +2124,12 @@
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
-          <t>Verbal quiz</t>
+          <t>Maths quiz</t>
         </is>
       </c>
       <c r="E11" s="7" t="inlineStr">
         <is>
-          <t>Random Verbal Reasoning round; answers and explanations withheld.</t>
+          <t>Random Maths round for a subtopic/topic and level in the student's programme; answers withheld.</t>
         </is>
       </c>
       <c r="F11" s="8" t="inlineStr">
@@ -2103,19 +2139,19 @@
       </c>
       <c r="G11" s="7" t="inlineStr">
         <is>
-          <t>src/app/api/vr/questions/route.ts</t>
+          <t>src/app/api/maths/questions/route.ts</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
         <is>
-          <t>Verbal</t>
+          <t>Maths</t>
         </is>
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>/api/vr/submit</t>
+          <t>/api/maths/submit</t>
         </is>
       </c>
       <c r="C12" s="7" t="inlineStr">
@@ -2125,12 +2161,12 @@
       </c>
       <c r="D12" s="7" t="inlineStr">
         <is>
-          <t>Verbal quiz</t>
+          <t>Maths quiz</t>
         </is>
       </c>
       <c r="E12" s="7" t="inlineStr">
         <is>
-          <t>Grades and saves a Verbal round.</t>
+          <t>Grades and saves a Maths round.</t>
         </is>
       </c>
       <c r="F12" s="8" t="inlineStr">
@@ -2140,19 +2176,19 @@
       </c>
       <c r="G12" s="7" t="inlineStr">
         <is>
-          <t>src/app/api/vr/submit/route.ts</t>
+          <t>src/app/api/maths/submit/route.ts</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
         <is>
-          <t>Non-Verbal</t>
+          <t>Verbal</t>
         </is>
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>/api/nvr/questions</t>
+          <t>/api/vr/questions</t>
         </is>
       </c>
       <c r="C13" s="7" t="inlineStr">
@@ -2162,12 +2198,12 @@
       </c>
       <c r="D13" s="7" t="inlineStr">
         <is>
-          <t>Non-Verbal quiz</t>
+          <t>Verbal quiz</t>
         </is>
       </c>
       <c r="E13" s="7" t="inlineStr">
         <is>
-          <t>Random Non-Verbal round with sanitised figures.</t>
+          <t>Random Verbal Reasoning round; answers and explanations withheld.</t>
         </is>
       </c>
       <c r="F13" s="8" t="inlineStr">
@@ -2177,19 +2213,19 @@
       </c>
       <c r="G13" s="7" t="inlineStr">
         <is>
-          <t>src/app/api/nvr/questions/route.ts</t>
+          <t>src/app/api/vr/questions/route.ts</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
         <is>
-          <t>Non-Verbal</t>
+          <t>Verbal</t>
         </is>
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>/api/nvr/submit</t>
+          <t>/api/vr/submit</t>
         </is>
       </c>
       <c r="C14" s="7" t="inlineStr">
@@ -2199,12 +2235,12 @@
       </c>
       <c r="D14" s="7" t="inlineStr">
         <is>
-          <t>Non-Verbal quiz</t>
+          <t>Verbal quiz</t>
         </is>
       </c>
       <c r="E14" s="7" t="inlineStr">
         <is>
-          <t>Grades and saves a Non-Verbal round.</t>
+          <t>Grades and saves a Verbal round.</t>
         </is>
       </c>
       <c r="F14" s="8" t="inlineStr">
@@ -2214,34 +2250,34 @@
       </c>
       <c r="G14" s="7" t="inlineStr">
         <is>
-          <t>src/app/api/nvr/submit/route.ts</t>
+          <t>src/app/api/vr/submit/route.ts</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
         <is>
-          <t>Review</t>
+          <t>Non-Verbal</t>
         </is>
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>/api/review/flag</t>
+          <t>/api/nvr/questions</t>
         </is>
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="D15" s="7" t="inlineStr">
         <is>
-          <t>Review pages (Maths, Verbal, Non-Verbal)</t>
+          <t>Non-Verbal quiz</t>
         </is>
       </c>
       <c r="E15" s="7" t="inlineStr">
         <is>
-          <t>Marks or unmarks a question as 'answer not clear' for an admin to check.</t>
+          <t>Random Non-Verbal round with sanitised figures.</t>
         </is>
       </c>
       <c r="F15" s="8" t="inlineStr">
@@ -2251,19 +2287,19 @@
       </c>
       <c r="G15" s="7" t="inlineStr">
         <is>
-          <t>src/app/api/review/flag/route.ts</t>
+          <t>src/app/api/nvr/questions/route.ts</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
         <is>
-          <t>Parent</t>
+          <t>Non-Verbal</t>
         </is>
       </c>
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>/api/parent/kids</t>
+          <t>/api/nvr/submit</t>
         </is>
       </c>
       <c r="C16" s="7" t="inlineStr">
@@ -2273,12 +2309,12 @@
       </c>
       <c r="D16" s="7" t="inlineStr">
         <is>
-          <t>Kids Profile</t>
+          <t>Non-Verbal quiz</t>
         </is>
       </c>
       <c r="E16" s="7" t="inlineStr">
         <is>
-          <t>Creates a child (STUDENT login) under the parent.</t>
+          <t>Grades and saves a Non-Verbal round.</t>
         </is>
       </c>
       <c r="F16" s="8" t="inlineStr">
@@ -2288,34 +2324,34 @@
       </c>
       <c r="G16" s="7" t="inlineStr">
         <is>
-          <t>src/app/api/parent/kids/route.ts</t>
+          <t>src/app/api/nvr/submit/route.ts</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
         <is>
-          <t>Parent</t>
+          <t>Review</t>
         </is>
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>/api/parent/kids/[studentId]</t>
+          <t>/api/review/flag</t>
         </is>
       </c>
       <c r="C17" s="7" t="inlineStr">
         <is>
-          <t>PUT, DELETE</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="D17" s="7" t="inlineStr">
         <is>
-          <t>Child profile page</t>
+          <t>Review pages (Maths, Verbal, Non-Verbal)</t>
         </is>
       </c>
       <c r="E17" s="7" t="inlineStr">
         <is>
-          <t>Updates or removes one of the parent's own children.</t>
+          <t>Marks or unmarks a question as 'answer not clear' for an admin to check.</t>
         </is>
       </c>
       <c r="F17" s="8" t="inlineStr">
@@ -2325,7 +2361,7 @@
       </c>
       <c r="G17" s="7" t="inlineStr">
         <is>
-          <t>src/app/api/parent/kids/[studentId]/route.ts</t>
+          <t>src/app/api/review/flag/route.ts</t>
         </is>
       </c>
     </row>
@@ -2337,22 +2373,22 @@
       </c>
       <c r="B18" s="7" t="inlineStr">
         <is>
-          <t>/api/parent/profile</t>
+          <t>/api/parent/kids</t>
         </is>
       </c>
       <c r="C18" s="7" t="inlineStr">
         <is>
-          <t>PUT</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="D18" s="7" t="inlineStr">
         <is>
-          <t>My Profile</t>
+          <t>Kids Profile</t>
         </is>
       </c>
       <c r="E18" s="7" t="inlineStr">
         <is>
-          <t>Saves the parent's own details.</t>
+          <t>Creates a child (STUDENT login) under the parent, with country and programme.</t>
         </is>
       </c>
       <c r="F18" s="8" t="inlineStr">
@@ -2362,7 +2398,7 @@
       </c>
       <c r="G18" s="7" t="inlineStr">
         <is>
-          <t>src/app/api/parent/profile/route.ts</t>
+          <t>src/app/api/parent/kids/route.ts</t>
         </is>
       </c>
     </row>
@@ -2374,22 +2410,22 @@
       </c>
       <c r="B19" s="7" t="inlineStr">
         <is>
-          <t>/api/parent/focus</t>
+          <t>/api/parent/kids/[studentId]</t>
         </is>
       </c>
       <c r="C19" s="7" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>PUT, DELETE</t>
         </is>
       </c>
       <c r="D19" s="7" t="inlineStr">
         <is>
-          <t>Practise this button (progress page)</t>
+          <t>Child profile page</t>
         </is>
       </c>
       <c r="E19" s="7" t="inlineStr">
         <is>
-          <t>Sets a topic as the child's focus, shown on the child's dashboard.</t>
+          <t>Updates (including programme) or removes one of the parent's own children.</t>
         </is>
       </c>
       <c r="F19" s="8" t="inlineStr">
@@ -2399,7 +2435,7 @@
       </c>
       <c r="G19" s="7" t="inlineStr">
         <is>
-          <t>src/app/api/parent/focus/route.ts</t>
+          <t>src/app/api/parent/kids/[studentId]/route.ts</t>
         </is>
       </c>
     </row>
@@ -2411,22 +2447,22 @@
       </c>
       <c r="B20" s="7" t="inlineStr">
         <is>
-          <t>/api/parent/focus/[focusId]</t>
+          <t>/api/parent/profile</t>
         </is>
       </c>
       <c r="C20" s="7" t="inlineStr">
         <is>
-          <t>PATCH</t>
+          <t>PUT</t>
         </is>
       </c>
       <c r="D20" s="7" t="inlineStr">
         <is>
-          <t>Remove link (progress page)</t>
+          <t>My Profile</t>
         </is>
       </c>
       <c r="E20" s="7" t="inlineStr">
         <is>
-          <t>Removes a focus from the child's dashboard; the row is kept with clearedAt set.</t>
+          <t>Saves the parent's own details.</t>
         </is>
       </c>
       <c r="F20" s="8" t="inlineStr">
@@ -2436,19 +2472,19 @@
       </c>
       <c r="G20" s="7" t="inlineStr">
         <is>
-          <t>src/app/api/parent/focus/[focusId]/route.ts</t>
+          <t>src/app/api/parent/profile/route.ts</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
         <is>
-          <t>Billing</t>
+          <t>Parent</t>
         </is>
       </c>
       <c r="B21" s="7" t="inlineStr">
         <is>
-          <t>/api/parent/billing/checkout</t>
+          <t>/api/parent/focus</t>
         </is>
       </c>
       <c r="C21" s="7" t="inlineStr">
@@ -2458,12 +2494,12 @@
       </c>
       <c r="D21" s="7" t="inlineStr">
         <is>
-          <t>Subscribe button</t>
+          <t>Practise this button (progress page)</t>
         </is>
       </c>
       <c r="E21" s="7" t="inlineStr">
         <is>
-          <t>Starts a monthly Stripe subscription for one child.</t>
+          <t>Sets a topic as the child's focus, shown on the child's dashboard.</t>
         </is>
       </c>
       <c r="F21" s="8" t="inlineStr">
@@ -2473,34 +2509,34 @@
       </c>
       <c r="G21" s="7" t="inlineStr">
         <is>
-          <t>src/app/api/parent/billing/checkout/route.ts</t>
+          <t>src/app/api/parent/focus/route.ts</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
         <is>
-          <t>Billing</t>
+          <t>Parent</t>
         </is>
       </c>
       <c r="B22" s="7" t="inlineStr">
         <is>
-          <t>/api/parent/billing/portal</t>
+          <t>/api/parent/focus/[focusId]</t>
         </is>
       </c>
       <c r="C22" s="7" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>PATCH</t>
         </is>
       </c>
       <c r="D22" s="7" t="inlineStr">
         <is>
-          <t>Manage billing button</t>
+          <t>Remove link (progress page)</t>
         </is>
       </c>
       <c r="E22" s="7" t="inlineStr">
         <is>
-          <t>Opens Stripe's billing portal (card, invoices, cancel).</t>
+          <t>Removes a focus from the child's dashboard; the row is kept with clearedAt set.</t>
         </is>
       </c>
       <c r="F22" s="8" t="inlineStr">
@@ -2510,7 +2546,7 @@
       </c>
       <c r="G22" s="7" t="inlineStr">
         <is>
-          <t>src/app/api/parent/billing/portal/route.ts</t>
+          <t>src/app/api/parent/focus/[focusId]/route.ts</t>
         </is>
       </c>
     </row>
@@ -2522,7 +2558,7 @@
       </c>
       <c r="B23" s="7" t="inlineStr">
         <is>
-          <t>/api/stripe/webhook</t>
+          <t>/api/parent/billing/checkout</t>
         </is>
       </c>
       <c r="C23" s="7" t="inlineStr">
@@ -2532,12 +2568,12 @@
       </c>
       <c r="D23" s="7" t="inlineStr">
         <is>
-          <t>Stripe</t>
+          <t>Subscribe button</t>
         </is>
       </c>
       <c r="E23" s="7" t="inlineStr">
         <is>
-          <t>Receives subscription events and updates the child's access.</t>
+          <t>Starts a monthly Stripe subscription for one child. Button currently hidden (src/config/billing.json).</t>
         </is>
       </c>
       <c r="F23" s="8" t="inlineStr">
@@ -2547,34 +2583,34 @@
       </c>
       <c r="G23" s="7" t="inlineStr">
         <is>
-          <t>src/app/api/stripe/webhook/route.ts</t>
+          <t>src/app/api/parent/billing/checkout/route.ts</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
         <is>
-          <t>Admin</t>
+          <t>Billing</t>
         </is>
       </c>
       <c r="B24" s="7" t="inlineStr">
         <is>
-          <t>/api/admin/english</t>
+          <t>/api/parent/billing/portal</t>
         </is>
       </c>
       <c r="C24" s="7" t="inlineStr">
         <is>
-          <t>GET, POST</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="D24" s="7" t="inlineStr">
         <is>
-          <t>Admin English</t>
+          <t>Manage billing button</t>
         </is>
       </c>
       <c r="E24" s="7" t="inlineStr">
         <is>
-          <t>Lists comprehensions (optionally by year) and creates new ones.</t>
+          <t>Opens Stripe's billing portal (card, invoices, cancel).</t>
         </is>
       </c>
       <c r="F24" s="8" t="inlineStr">
@@ -2584,19 +2620,19 @@
       </c>
       <c r="G24" s="7" t="inlineStr">
         <is>
-          <t>src/app/api/admin/english/route.ts</t>
+          <t>src/app/api/parent/billing/portal/route.ts</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
         <is>
-          <t>Admin</t>
+          <t>Billing</t>
         </is>
       </c>
       <c r="B25" s="7" t="inlineStr">
         <is>
-          <t>/api/admin/english/generate</t>
+          <t>/api/stripe/webhook</t>
         </is>
       </c>
       <c r="C25" s="7" t="inlineStr">
@@ -2606,12 +2642,12 @@
       </c>
       <c r="D25" s="7" t="inlineStr">
         <is>
-          <t>Admin English</t>
+          <t>Stripe</t>
         </is>
       </c>
       <c r="E25" s="7" t="inlineStr">
         <is>
-          <t>Drafts a comprehension with Claude for the admin to review; saves nothing.</t>
+          <t>Receives subscription events and updates the child's access.</t>
         </is>
       </c>
       <c r="F25" s="8" t="inlineStr">
@@ -2621,7 +2657,7 @@
       </c>
       <c r="G25" s="7" t="inlineStr">
         <is>
-          <t>src/app/api/admin/english/generate/route.ts</t>
+          <t>src/app/api/stripe/webhook/route.ts</t>
         </is>
       </c>
     </row>
@@ -2633,12 +2669,12 @@
       </c>
       <c r="B26" s="7" t="inlineStr">
         <is>
-          <t>/api/admin/comps/[compId]</t>
+          <t>/api/admin/english</t>
         </is>
       </c>
       <c r="C26" s="7" t="inlineStr">
         <is>
-          <t>GET, PATCH, DELETE</t>
+          <t>GET, POST</t>
         </is>
       </c>
       <c r="D26" s="7" t="inlineStr">
@@ -2648,7 +2684,7 @@
       </c>
       <c r="E26" s="7" t="inlineStr">
         <is>
-          <t>Reads, edits or removes one comprehension.</t>
+          <t>Lists comprehensions (optionally by year) and creates new ones.</t>
         </is>
       </c>
       <c r="F26" s="8" t="inlineStr">
@@ -2658,7 +2694,7 @@
       </c>
       <c r="G26" s="7" t="inlineStr">
         <is>
-          <t>src/app/api/admin/comps/[compId]/route.ts</t>
+          <t>src/app/api/admin/english/route.ts</t>
         </is>
       </c>
     </row>
@@ -2670,7 +2706,7 @@
       </c>
       <c r="B27" s="7" t="inlineStr">
         <is>
-          <t>/api/admin/comps/[compId]/questions</t>
+          <t>/api/admin/english/generate</t>
         </is>
       </c>
       <c r="C27" s="7" t="inlineStr">
@@ -2685,7 +2721,7 @@
       </c>
       <c r="E27" s="7" t="inlineStr">
         <is>
-          <t>Adds questions to a comprehension.</t>
+          <t>Drafts a comprehension with Claude (Opus 5.5) from prompt, level, reference passages and copyright guidance; saves nothing.</t>
         </is>
       </c>
       <c r="F27" s="8" t="inlineStr">
@@ -2695,7 +2731,7 @@
       </c>
       <c r="G27" s="7" t="inlineStr">
         <is>
-          <t>src/app/api/admin/comps/[compId]/questions/route.ts</t>
+          <t>src/app/api/admin/english/generate/route.ts</t>
         </is>
       </c>
     </row>
@@ -2707,12 +2743,12 @@
       </c>
       <c r="B28" s="7" t="inlineStr">
         <is>
-          <t>/api/admin/comps/[compId]/questions/[questionId]</t>
+          <t>/api/admin/comps/[compId]</t>
         </is>
       </c>
       <c r="C28" s="7" t="inlineStr">
         <is>
-          <t>PATCH, DELETE</t>
+          <t>GET, PATCH, DELETE</t>
         </is>
       </c>
       <c r="D28" s="7" t="inlineStr">
@@ -2722,7 +2758,7 @@
       </c>
       <c r="E28" s="7" t="inlineStr">
         <is>
-          <t>Edits or removes one comprehension question.</t>
+          <t>Reads, edits or removes one comprehension.</t>
         </is>
       </c>
       <c r="F28" s="8" t="inlineStr">
@@ -2732,7 +2768,7 @@
       </c>
       <c r="G28" s="7" t="inlineStr">
         <is>
-          <t>src/app/api/admin/comps/[compId]/questions/[questionId]/route.ts</t>
+          <t>src/app/api/admin/comps/[compId]/route.ts</t>
         </is>
       </c>
     </row>
@@ -2744,7 +2780,7 @@
       </c>
       <c r="B29" s="7" t="inlineStr">
         <is>
-          <t>/api/admin/refresh-question-bank</t>
+          <t>/api/admin/comps/[compId]/questions</t>
         </is>
       </c>
       <c r="C29" s="7" t="inlineStr">
@@ -2754,12 +2790,12 @@
       </c>
       <c r="D29" s="7" t="inlineStr">
         <is>
-          <t>Admin home Refresh now button</t>
+          <t>Admin English</t>
         </is>
       </c>
       <c r="E29" s="7" t="inlineStr">
         <is>
-          <t>Clears the cached Maths, Verbal and Non-Verbal level/topic lists (otherwise flushed daily at 03:00 UK time).</t>
+          <t>Adds questions to a comprehension.</t>
         </is>
       </c>
       <c r="F29" s="8" t="inlineStr">
@@ -2769,7 +2805,7 @@
       </c>
       <c r="G29" s="7" t="inlineStr">
         <is>
-          <t>src/app/api/admin/refresh-question-bank/route.ts</t>
+          <t>src/app/api/admin/comps/[compId]/questions/route.ts</t>
         </is>
       </c>
     </row>
@@ -2781,22 +2817,22 @@
       </c>
       <c r="B30" s="7" t="inlineStr">
         <is>
-          <t>/api/admin/parent-password</t>
+          <t>/api/admin/comps/[compId]/questions/[questionId]</t>
         </is>
       </c>
       <c r="C30" s="7" t="inlineStr">
         <is>
-          <t>GET, POST</t>
+          <t>PATCH, DELETE</t>
         </is>
       </c>
       <c r="D30" s="7" t="inlineStr">
         <is>
-          <t>Admin parent-password page</t>
+          <t>Admin English</t>
         </is>
       </c>
       <c r="E30" s="7" t="inlineStr">
         <is>
-          <t>Lists parents and resets a parent's password.</t>
+          <t>Edits or removes one comprehension question.</t>
         </is>
       </c>
       <c r="F30" s="8" t="inlineStr">
@@ -2806,7 +2842,7 @@
       </c>
       <c r="G30" s="7" t="inlineStr">
         <is>
-          <t>src/app/api/admin/parent-password/route.ts</t>
+          <t>src/app/api/admin/comps/[compId]/questions/[questionId]/route.ts</t>
         </is>
       </c>
     </row>
@@ -2818,37 +2854,652 @@
       </c>
       <c r="B31" s="7" t="inlineStr">
         <is>
+          <t>/api/admin/refresh-question-bank</t>
+        </is>
+      </c>
+      <c r="C31" s="7" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="D31" s="7" t="inlineStr">
+        <is>
+          <t>Admin home Refresh now button</t>
+        </is>
+      </c>
+      <c r="E31" s="7" t="inlineStr">
+        <is>
+          <t>Clears the cached Maths, Verbal and Non-Verbal level/topic lists (otherwise flushed daily at 03:00 UK time).</t>
+        </is>
+      </c>
+      <c r="F31" s="8" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="G31" s="7" t="inlineStr">
+        <is>
+          <t>src/app/api/admin/refresh-question-bank/route.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="7" t="inlineStr">
+        <is>
+          <t>Admin</t>
+        </is>
+      </c>
+      <c r="B32" s="7" t="inlineStr">
+        <is>
+          <t>/api/admin/parent-password</t>
+        </is>
+      </c>
+      <c r="C32" s="7" t="inlineStr">
+        <is>
+          <t>GET, POST</t>
+        </is>
+      </c>
+      <c r="D32" s="7" t="inlineStr">
+        <is>
+          <t>Admin parent-password page</t>
+        </is>
+      </c>
+      <c r="E32" s="7" t="inlineStr">
+        <is>
+          <t>Lists parents and resets a parent's password.</t>
+        </is>
+      </c>
+      <c r="F32" s="8" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="G32" s="7" t="inlineStr">
+        <is>
+          <t>src/app/api/admin/parent-password/route.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="7" t="inlineStr">
+        <is>
+          <t>Admin</t>
+        </is>
+      </c>
+      <c r="B33" s="7" t="inlineStr">
+        <is>
           <t>/api/admin/admin-password</t>
         </is>
       </c>
-      <c r="C31" s="7" t="inlineStr">
+      <c r="C33" s="7" t="inlineStr">
         <is>
           <t>GET, POST</t>
         </is>
       </c>
-      <c r="D31" s="7" t="inlineStr">
+      <c r="D33" s="7" t="inlineStr">
         <is>
           <t>Admin admin-password page</t>
         </is>
       </c>
-      <c r="E31" s="7" t="inlineStr">
+      <c r="E33" s="7" t="inlineStr">
         <is>
           <t>Lists admins and resets an admin's password.</t>
         </is>
       </c>
-      <c r="F31" s="8" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-      <c r="G31" s="7" t="inlineStr">
+      <c r="F33" s="8" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="G33" s="7" t="inlineStr">
         <is>
           <t>src/app/api/admin/admin-password/route.ts</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G31"/>
+  <autoFilter ref="A1:G33"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="80" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>File</t>
+        </is>
+      </c>
+      <c r="B1" s="6" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
+      <c r="C1" s="6" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="D1" s="6" t="inlineStr">
+        <is>
+          <t>What it controls</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>src/config/progress.json</t>
+        </is>
+      </c>
+      <c r="B2" s="7" t="inlineStr">
+        <is>
+          <t>targetPercent</t>
+        </is>
+      </c>
+      <c r="C2" s="7" t="inlineStr">
+        <is>
+          <t>75</t>
+        </is>
+      </c>
+      <c r="D2" s="7" t="inlineStr">
+        <is>
+          <t>Dashed target line on the parent's score bars and the start of green.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>src/config/progress.json</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>amberFromPercent</t>
+        </is>
+      </c>
+      <c r="C3" s="7" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="D3" s="7" t="inlineStr">
+        <is>
+          <t>Amber runs from here to the target; below it is red.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>src/config/progress.json</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>minAnswers</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>Fewer answers than this: faded grey bar, left out of Focus next.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>src/config/progress.json</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>focusCount</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>How many topics Focus next suggests.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>src/config/progress.json</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>trendDays</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>Trend arrow compares the score now with this many days ago.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>src/config/progress.json</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>englishSkillFamilies</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>4 families</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>Groups English question types (Finding information, Vocabulary, Order of events, Deeper understanding).</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>src/config/session.json</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>idleTimeoutMinutes</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>150</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>Sign-out after this long with no activity.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>src/config/session.json</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>warningSeconds</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>'Still there?' box appears this long before sign-out.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>src/config/session.json</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>keepaliveEveryMinutes</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>Session renewed at most this often while active.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>src/config/security.json</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>login.maxFailuresPerAccount</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>Wrong passwords before a login ID is locked.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>src/config/security.json</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>login.lockoutMinutes</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="D12" s="7" t="inlineStr">
+        <is>
+          <t>How long a login ID stays locked.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>src/config/security.json</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>login.maxAttemptsPerIp</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="D13" s="7" t="inlineStr">
+        <is>
+          <t>Login attempts per network address per window.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>src/config/security.json</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>register / forgotPassword / resetPassword</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>5/h, 5/15m, 10/15m</t>
+        </is>
+      </c>
+      <c r="D14" s="7" t="inlineStr">
+        <is>
+          <t>Requests per network address.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>src/config/billing.json</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>showSubscribeButton</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="D15" s="7" t="inlineStr">
+        <is>
+          <t>Hides the Subscribe button and 'Not subscribed' chip on the parent dashboard.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:D15"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="90" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>File (prisma/sql)</t>
+        </is>
+      </c>
+      <c r="B1" s="6" t="inlineStr">
+        <is>
+          <t>What it does</t>
+        </is>
+      </c>
+      <c r="C1" s="6" t="inlineStr">
+        <is>
+          <t>Must run before deploy?</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>024_terms_acceptance.sql</t>
+        </is>
+      </c>
+      <c r="B2" s="7" t="inlineStr">
+        <is>
+          <t>userProfile.termsAcceptedAt: when a parent accepted the Terms.</t>
+        </is>
+      </c>
+      <c r="C2" s="7" t="inlineStr">
+        <is>
+          <t>Yes - login fails without it</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>025_flag_unclear_maths.sql</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>'Answer not clear' flag columns on testTrackerMath.</t>
+        </is>
+      </c>
+      <c r="C3" s="7" t="inlineStr">
+        <is>
+          <t>Yes - Maths review pages</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>026_bigint_ids.sql</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>Every id and foreign key INTEGER to BIGINT, plus id sequences.</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>027_drop_legacy_tables.sql</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>Drops unused Day, Question, Attempt, Answer tables. Take a backup first.</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>028_student_focus.sql</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>studentFocus table for Practise this / Your focus this week.</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>Yes - parent progress and student dashboard</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>029_nvr_why_wrong.sql</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>whyWrongA-E columns on gsNvrQuestions.</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>Yes - Non-Verbal review pages</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>030_nvr_text_options.sql</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>Allows optionFormat 'text' for Non-Verbal letter-code options.</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>Yes - before inserting text-option questions</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>031_country.sql</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>country table (249 countries with dialling codes) and userProfile.countryCode.</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>Yes - sign-up and add-child</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>032_programme.sql</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>programme table (Grammar School active; GCSE, A-Level inactive) and programmeCode on users and all four question banks.</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>Yes - login fails without it</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:C10"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>